<commit_message>
Configure for Render deployment and secure API keys
</commit_message>
<xml_diff>
--- a/notebooks/segmentation result.xlsx
+++ b/notebooks/segmentation result.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="22527"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\OutlesClassifier-ChatAssist\notebooks\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1C5CE39-8FD0-434C-8FCC-B3FF29D42309}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,10 +24,100 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+  <si>
+    <t>Cluster</t>
+  </si>
+  <si>
+    <t>Segment Name</t>
+  </si>
+  <si>
+    <t>Key Characteristics</t>
+  </si>
+  <si>
+    <t>Total Sales</t>
+  </si>
+  <si>
+    <t>Unique Products</t>
+  </si>
+  <si>
+    <t>Avg Sales / Product</t>
+  </si>
+  <si>
+    <t>Total Pieces</t>
+  </si>
+  <si>
+    <t>Total KG/Litre</t>
+  </si>
+  <si>
+    <t>Outlet Class Mix</t>
+  </si>
+  <si>
+    <t>Mid-Value Balanced Outlets</t>
+  </si>
+  <si>
+    <t>Moderate sales, decent product variety, general-purpose outlets, not highly specialized</t>
+  </si>
+  <si>
+    <t>C (43.54%), D (27.34%), B (17.35%), A (11.77%)</t>
+  </si>
+  <si>
+    <t>Low-Value Efficient Outlets</t>
+  </si>
+  <si>
+    <t>Smaller outlets, fewer products, but high efficiency per product; focused selling</t>
+  </si>
+  <si>
+    <t>D (44.48%), C (38.10%), B (10.52%), A (6.88%)</t>
+  </si>
+  <si>
+    <t>Ultra-Premium Niche Accounts</t>
+  </si>
+  <si>
+    <t>Extremely high sales, massive transactions, niche or bulk specialists, very high impact</t>
+  </si>
+  <si>
+    <t>A (80.00%), C (10.00%), D (10.00%)</t>
+  </si>
+  <si>
+    <t>Elite High-Value Performers</t>
+  </si>
+  <si>
+    <t>High sales + strong product mix, consistent top performers, large-scale outlets</t>
+  </si>
+  <si>
+    <t>A (83.53%), D (9.41%), 
+B (3.53%), 
+C (3.53%)</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="3">
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="173" formatCode="&quot;₹&quot;\ #,##0"/>
+    <numFmt numFmtId="174" formatCode="0.0"/>
+  </numFmts>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -46,13 +142,42 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="173" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="174" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -330,10 +455,165 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.42578125" style="9"/>
+    <col min="2" max="2" width="20.7109375" style="7" customWidth="1"/>
+    <col min="3" max="3" width="21.85546875" style="7" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" style="7" customWidth="1"/>
+    <col min="5" max="7" width="11.42578125" style="7"/>
+    <col min="8" max="8" width="11.42578125" style="7" customWidth="1"/>
+    <col min="9" max="16384" width="11.42578125" style="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+      <c r="A2" s="8">
+        <v>0</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="5">
+        <v>63350.95</v>
+      </c>
+      <c r="E2" s="2">
+        <v>22.38</v>
+      </c>
+      <c r="F2" s="4">
+        <v>1586.17</v>
+      </c>
+      <c r="G2" s="2">
+        <v>733.26</v>
+      </c>
+      <c r="H2" s="6">
+        <v>396.93</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A3" s="8">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="5">
+        <v>25616.11</v>
+      </c>
+      <c r="E3" s="2">
+        <v>8.15</v>
+      </c>
+      <c r="F3" s="4">
+        <v>2025.99</v>
+      </c>
+      <c r="G3" s="2">
+        <v>257.08</v>
+      </c>
+      <c r="H3" s="6">
+        <v>155.41999999999999</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+      <c r="A4" s="8">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="5">
+        <v>14016689.140000001</v>
+      </c>
+      <c r="E4" s="2">
+        <v>11.3</v>
+      </c>
+      <c r="F4" s="4">
+        <v>837754</v>
+      </c>
+      <c r="G4" s="4">
+        <v>98390</v>
+      </c>
+      <c r="H4" s="6">
+        <v>108569.89</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+      <c r="A5" s="8">
+        <v>3</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="5">
+        <v>3152058.4</v>
+      </c>
+      <c r="E5" s="2">
+        <v>14.68</v>
+      </c>
+      <c r="F5" s="4">
+        <v>137210.43</v>
+      </c>
+      <c r="G5" s="4">
+        <v>23819.21</v>
+      </c>
+      <c r="H5" s="6">
+        <v>17630.95</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>